<commit_message>
Testing to avg yield
</commit_message>
<xml_diff>
--- a/data/WHO_HTS_Multipliers.xlsx
+++ b/data/WHO_HTS_Multipliers.xlsx
@@ -8,20 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_DE3F3E6CDD7A619BF436840F588153E29DC84B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="11_DE3F3E6CDD7A619BF436840F588153E29DC84B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{260D533D-A0D4-6F49-8DDF-4CDCC9D9BA9B}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="14380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="940" windowWidth="28800" windowHeight="14380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HTS Multipliers" sheetId="1" r:id="rId1"/>
     <sheet name="Multiplier Summary" sheetId="2" r:id="rId2"/>
+    <sheet name="Tier testing" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'HTS Multipliers'!$A$1:$BY$37</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="78">
   <si>
     <t>Country</t>
   </si>
@@ -213,6 +217,48 @@
   </si>
   <si>
     <t>≥2x countries</t>
+  </si>
+  <si>
+    <t>ANC HIV testing</t>
+  </si>
+  <si>
+    <t>EID</t>
+  </si>
+  <si>
+    <t>HIVST (Community)</t>
+  </si>
+  <si>
+    <t>HIVST (Facility)</t>
+  </si>
+  <si>
+    <t>PNC HIV testing</t>
+  </si>
+  <si>
+    <t>Community-based testing</t>
+  </si>
+  <si>
+    <t>Facility-based testing (general)</t>
+  </si>
+  <si>
+    <t>Facility-based testing (targeted)</t>
+  </si>
+  <si>
+    <t>Key populations &amp; STI testing</t>
+  </si>
+  <si>
+    <t>Network/Index testing</t>
+  </si>
+  <si>
+    <t>Tier</t>
+  </si>
+  <si>
+    <t>HTS dashboard</t>
+  </si>
+  <si>
+    <t>HTS breakdowns possible</t>
+  </si>
+  <si>
+    <t>Facility PITC + Facility VCT</t>
   </si>
 </sst>
 </file>
@@ -223,7 +269,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -243,6 +289,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -275,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -308,6 +362,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -604,6 +664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:BY37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -844,7 +905,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:77" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:77" ht="28" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1077,7 +1138,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1173,7 +1234,7 @@
       <c r="BW3" s="8"/>
       <c r="BX3" s="4"/>
     </row>
-    <row r="4" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
@@ -1376,7 +1437,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="5" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1597,7 +1658,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="6" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
@@ -1820,7 +1881,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="7" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>26</v>
       </c>
@@ -1969,7 +2030,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="8" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -2108,7 +2169,7 @@
       <c r="BX8" s="3"/>
       <c r="BY8" s="2"/>
     </row>
-    <row r="9" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -2233,7 +2294,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="10" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>29</v>
       </c>
@@ -2436,7 +2497,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="11" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -2597,7 +2658,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="12" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>31</v>
       </c>
@@ -2806,7 +2867,7 @@
       <c r="BX12" s="3"/>
       <c r="BY12" s="2"/>
     </row>
-    <row r="13" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -3119,7 +3180,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="15" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -3335,7 +3396,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="16" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>35</v>
       </c>
@@ -3518,7 +3579,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="17" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -3655,7 +3716,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="18" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>37</v>
       </c>
@@ -3888,7 +3949,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="19" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -4109,7 +4170,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="20" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
@@ -4302,7 +4363,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="21" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>40</v>
       </c>
@@ -4446,7 +4507,7 @@
       <c r="BW21" s="8"/>
       <c r="BX21" s="4"/>
     </row>
-    <row r="22" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>41</v>
       </c>
@@ -4629,7 +4690,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="23" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -4862,7 +4923,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="24" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>43</v>
       </c>
@@ -5075,7 +5136,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="25" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>44</v>
       </c>
@@ -5296,7 +5357,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="26" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>45</v>
       </c>
@@ -5409,7 +5470,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="27" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>46</v>
       </c>
@@ -5630,7 +5691,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="28" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>47</v>
       </c>
@@ -5753,7 +5814,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="29" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>48</v>
       </c>
@@ -5902,7 +5963,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="30" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>49</v>
       </c>
@@ -6125,7 +6186,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="31" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>50</v>
       </c>
@@ -6209,7 +6270,7 @@
       <c r="BW31" s="8"/>
       <c r="BX31" s="4"/>
     </row>
-    <row r="32" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>51</v>
       </c>
@@ -6298,7 +6359,7 @@
       <c r="BX32" s="3"/>
       <c r="BY32" s="2"/>
     </row>
-    <row r="33" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>52</v>
       </c>
@@ -6466,7 +6527,7 @@
       <c r="BW33" s="8"/>
       <c r="BX33" s="4"/>
     </row>
-    <row r="34" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>53</v>
       </c>
@@ -6609,7 +6670,7 @@
       <c r="BX34" s="3"/>
       <c r="BY34" s="2"/>
     </row>
-    <row r="35" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>54</v>
       </c>
@@ -6763,7 +6824,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="36" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>55</v>
       </c>
@@ -6896,7 +6957,7 @@
       <c r="BX36" s="3"/>
       <c r="BY36" s="2"/>
     </row>
-    <row r="37" spans="1:77" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:77" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>56</v>
       </c>
@@ -6947,23 +7008,90 @@
       <c r="BX37" s="4"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:BY37" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="ZAF"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1" showButton="0"/>
+    <filterColumn colId="2" showButton="0"/>
+    <filterColumn colId="3" showButton="0"/>
+    <filterColumn colId="5" showButton="0"/>
+    <filterColumn colId="6" showButton="0"/>
+    <filterColumn colId="7" showButton="0"/>
+    <filterColumn colId="8" showButton="0"/>
+    <filterColumn colId="10" showButton="0"/>
+    <filterColumn colId="11" showButton="0"/>
+    <filterColumn colId="12" showButton="0"/>
+    <filterColumn colId="13" showButton="0"/>
+    <filterColumn colId="15" showButton="0"/>
+    <filterColumn colId="16" showButton="0"/>
+    <filterColumn colId="17" showButton="0"/>
+    <filterColumn colId="18" showButton="0"/>
+    <filterColumn colId="20" showButton="0"/>
+    <filterColumn colId="21" showButton="0"/>
+    <filterColumn colId="22" showButton="0"/>
+    <filterColumn colId="23" showButton="0"/>
+    <filterColumn colId="25" showButton="0"/>
+    <filterColumn colId="26" showButton="0"/>
+    <filterColumn colId="27" showButton="0"/>
+    <filterColumn colId="28" showButton="0"/>
+    <filterColumn colId="30" showButton="0"/>
+    <filterColumn colId="31" showButton="0"/>
+    <filterColumn colId="32" showButton="0"/>
+    <filterColumn colId="33" showButton="0"/>
+    <filterColumn colId="35" showButton="0"/>
+    <filterColumn colId="36" showButton="0"/>
+    <filterColumn colId="37" showButton="0"/>
+    <filterColumn colId="38" showButton="0"/>
+    <filterColumn colId="40" showButton="0"/>
+    <filterColumn colId="41" showButton="0"/>
+    <filterColumn colId="42" showButton="0"/>
+    <filterColumn colId="43" showButton="0"/>
+    <filterColumn colId="45" showButton="0"/>
+    <filterColumn colId="46" showButton="0"/>
+    <filterColumn colId="47" showButton="0"/>
+    <filterColumn colId="48" showButton="0"/>
+    <filterColumn colId="50" showButton="0"/>
+    <filterColumn colId="51" showButton="0"/>
+    <filterColumn colId="52" showButton="0"/>
+    <filterColumn colId="53" showButton="0"/>
+    <filterColumn colId="55" showButton="0"/>
+    <filterColumn colId="56" showButton="0"/>
+    <filterColumn colId="57" showButton="0"/>
+    <filterColumn colId="58" showButton="0"/>
+    <filterColumn colId="60" showButton="0"/>
+    <filterColumn colId="61" showButton="0"/>
+    <filterColumn colId="62" showButton="0"/>
+    <filterColumn colId="63" showButton="0"/>
+    <filterColumn colId="65" showButton="0"/>
+    <filterColumn colId="66" showButton="0"/>
+    <filterColumn colId="67" showButton="0"/>
+    <filterColumn colId="68" showButton="0"/>
+    <filterColumn colId="70" showButton="0"/>
+    <filterColumn colId="71" showButton="0"/>
+    <filterColumn colId="72" showButton="0"/>
+    <filterColumn colId="73" showButton="0"/>
+    <filterColumn colId="75" showButton="0"/>
+  </autoFilter>
   <mergeCells count="16">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="P1:T1"/>
+    <mergeCell ref="U1:Y1"/>
+    <mergeCell ref="Z1:AD1"/>
+    <mergeCell ref="AE1:AI1"/>
+    <mergeCell ref="AJ1:AN1"/>
+    <mergeCell ref="AO1:AS1"/>
+    <mergeCell ref="AT1:AX1"/>
     <mergeCell ref="BX1:BY1"/>
     <mergeCell ref="AY1:BC1"/>
     <mergeCell ref="BD1:BH1"/>
     <mergeCell ref="BI1:BM1"/>
     <mergeCell ref="BN1:BR1"/>
     <mergeCell ref="BS1:BW1"/>
-    <mergeCell ref="Z1:AD1"/>
-    <mergeCell ref="AE1:AI1"/>
-    <mergeCell ref="AJ1:AN1"/>
-    <mergeCell ref="AO1:AS1"/>
-    <mergeCell ref="AT1:AX1"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:O1"/>
-    <mergeCell ref="P1:T1"/>
-    <mergeCell ref="U1:Y1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -7340,4 +7468,162 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{357BE56B-82BE-5547-9AD2-3D1E5961D327}">
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="G3" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="13"/>
+      <c r="G4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G5" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E6" s="14"/>
+      <c r="G6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="15"/>
+      <c r="G7" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E8" s="14"/>
+      <c r="G8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="15"/>
+      <c r="G9" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E10" s="14"/>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="15"/>
+      <c r="G11" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E12" s="14"/>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="15"/>
+      <c r="G13" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E14" s="14"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="15"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="E16" s="14"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E17" s="15"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" s="14"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E19" s="14"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:B4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>